<commit_message>
feat(F-NAR-016): TREE-DIF-052 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-052.xlsx
+++ b/stories/arbres/TREE-DIF-052.xlsx
@@ -1378,12 +1378,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Près du sac, la clochette attend. Le seau bleu dort, vide. La pelle jaune est posée. Tu prends quoi d'abord, Mila ?</t>
+          <t>Avant de sortir, trois affaires attendent. La clochette, le seau bleu, la pelle jaune. Tu prends quoi d'abord, Mila ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Près du sac, la clochette attend. Le seau bleu dort, vide. La pelle jaune est posée. Tu prends quoi d'abord, Mila ?</t>
+          <t>Avant de sortir, trois affaires attendent. La clochette, le seau bleu, la pelle jaune. Tu prends quoi d'abord, Mila ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1542,9 +1542,8 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Près du sac, la clochette attend.
-narrateur|Le seau bleu dort, vide.
-narrateur|La pelle jaune est posée.
+          <t>narrateur|Avant de sortir, trois affaires attendent.
+narrateur|La clochette, le seau bleu, la pelle jaune.
 maman|Tu prends quoi d'abord, Mila ?</t>
         </is>
       </c>
@@ -2675,12 +2674,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Sarah essuie, puis reprend le bord de la cloche. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
+          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Puis elle reprend le bord de la cloche. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Sarah essuie, puis reprend le bord de la cloche. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
+          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Puis elle reprend le bord de la cloche. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2818,7 +2817,7 @@
           <t>enfant-f|Maman, le torchon, s'il te plaît.
 maman|Tiens, tout doux, sur les verres.
 narrateur|Sarah frotte un rond, puis un autre.
-narrateur|Sarah essuie, puis reprend le bord de la cloche.
+narrateur|Puis elle reprend le bord de la cloche.
 copine|Je vois les coquillages !
 enfant-f|Le rose est à toi, maintenant.
 narrateur|Les lunettes rendent le rocher tout net.
@@ -2850,12 +2849,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La clochette rentre, encore salée. Une goutte reste sur un coquillage, ronde. On rentre, Sarah. La jetée redevient calme.</t>
+          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La clochette rentre, encore salée. Le phare tient sur la jetée. On rentre, Sarah. La jetée redevient calme.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La clochette rentre, encore salée. Une goutte reste sur un coquillage, ronde. On rentre, Sarah. La jetée redevient calme.</t>
+          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La clochette rentre, encore salée. Le phare tient sur la jetée. On rentre, Sarah. La jetée redevient calme.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2996,7 +2995,7 @@
 papa|Vous avez bâti, chacune avec sa vue.
 maman|Le bois sèche déjà, tout doux.
 narrateur|La clochette rentre, encore salée.
-narrateur|Une goutte reste sur un coquillage, ronde.
+narrateur|Le phare tient sur la jetée.
 enfant-f|On rentre, Sarah.
 narrateur|La jetée redevient calme.</t>
         </is>
@@ -3200,12 +3199,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La clochette rentre, encore salée. Une ombre de coquillage reste au fond. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
+          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La clochette rentre, encore salée. Le phare tient, encore un peu flou. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La clochette rentre, encore salée. Une ombre de coquillage reste au fond. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
+          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La clochette rentre, encore salée. Le phare tient, encore un peu flou. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3346,7 +3345,7 @@
 papa|Les verres flous n'ont pas arrêté le phare.
 maman|La jetée se tait, enfin.
 narrateur|La clochette rentre, encore salée.
-narrateur|Une ombre de coquillage reste au fond.
+narrateur|Le phare tient, encore un peu flou.
 enfant-f|À demain, le rocher.
 narrateur|Le rebord redevient tiède, déjà.</t>
         </is>
@@ -3550,12 +3549,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La clochette rentre, encore salée. Mila souffle sur un coquillage, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
+          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La clochette rentre, encore salée. Mila souffle sur le phare, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La clochette rentre, encore salée. Mila souffle sur un coquillage, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
+          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La clochette rentre, encore salée. Mila souffle sur le phare, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3696,7 +3695,7 @@
 maman|Le pas en arrière a rendu les coquillages.
 papa|Vous avez laissé le temps aux lunettes.
 narrateur|La clochette rentre, encore salée.
-narrateur|Mila souffle sur un coquillage, tout léger.
+narrateur|Mila souffle sur le phare, tout léger.
 copine|Il brille encore.
 narrateur|Le bois reprend, plus loin.</t>
         </is>
@@ -4271,12 +4270,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La clochette rentre, encore salée. Une mèche sèche contre le col, tout calme. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
+          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La clochette rentre, encore salée. Le phare tient sur la dune. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La clochette rentre, encore salée. Une mèche sèche contre le col, tout calme. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
+          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La clochette rentre, encore salée. Le phare tient sur la dune. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4417,7 +4416,7 @@
 papa|Chacune a eu sa hauteur, sous le vent.
 maman|Le sable sèche déjà.
 narrateur|La clochette rentre, encore salée.
-narrateur|Une mèche sèche contre le col, tout calme.
+narrateur|Le phare tient sur la dune.
 enfant-f|On rentre, la dune reste.
 narrateur|Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
@@ -4621,12 +4620,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La clochette rentre, encore salée. Mila souffle dessus, tout léger. Elle part. Le sel s'efface déjà du sable.</t>
+          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La clochette rentre, encore salée. Le phare tient, encore salé. Il reste. Le sel s'efface déjà du sable.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La clochette rentre, encore salée. Mila souffle dessus, tout léger. Elle part. Le sel s'efface déjà du sable.</t>
+          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La clochette rentre, encore salée. Le phare tient, encore salé. Il reste. Le sel s'efface déjà du sable.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4767,8 +4766,8 @@
 maman|L'eau des cheveux s'en est allée.
 papa|La dune vous rend le silence.
 narrateur|La clochette rentre, encore salée.
-narrateur|Mila souffle dessus, tout léger.
-copine|Elle part.
+narrateur|Le phare tient, encore salé.
+copine|Il reste.
 narrateur|Le sel s'efface déjà du sable.</t>
         </is>
       </c>
@@ -4971,12 +4970,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La clochette rentre, encore salée. Un rebord vide attend, tout bas. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
+          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La clochette rentre, encore salée. Le phare reste, tout petit. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La clochette rentre, encore salée. Un rebord vide attend, tout bas. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
+          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La clochette rentre, encore salée. Le phare reste, tout petit. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5117,7 +5116,7 @@
 papa|Vous avez bâti avec ce que vous aviez.
 maman|Les cheveux n'avaient plus besoin d'être pris.
 narrateur|La clochette rentre, encore salée.
-narrateur|Un rebord vide attend, tout bas.
+narrateur|Le phare reste, tout petit.
 enfant-f|On se dit au revoir, dune.
 narrateur|Les chaussons glissent vers la maison.</t>
         </is>
@@ -5692,12 +5691,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La clochette rentre, encore salée. Un coquillage rose reste sur le bois. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
+          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La clochette rentre, encore salée. Le phare tient dans l'écume. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La clochette rentre, encore salée. Un coquillage rose reste sur le bois. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
+          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La clochette rentre, encore salée. Le phare tient dans l'écume. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5838,7 +5837,7 @@
 papa|Les manches ont laissé les coquillages passer.
 maman|L'écume redevient de l'eau, tout simple.
 narrateur|La clochette rentre, encore salée.
-narrateur|Un coquillage rose reste sur le bois.
+narrateur|Le phare tient dans l'écume.
 enfant-f|On rentre, Sarah.
 narrateur|L'écume reprend sa forme, tout lente.</t>
         </is>
@@ -6042,12 +6041,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La clochette rentre, encore salée. Mila lisse un coquillage, tout doux. Il a bien roulé. La vague reprend son calme, déjà.</t>
+          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La clochette rentre, encore salée. Mila lisse le phare, tout doux. Il a bien tenu. La vague reprend son calme, déjà.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La clochette rentre, encore salée. Mila lisse un coquillage, tout doux. Il a bien roulé. La vague reprend son calme, déjà.</t>
+          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La clochette rentre, encore salée. Mila lisse le phare, tout doux. Il a bien tenu. La vague reprend son calme, déjà.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6188,8 +6187,8 @@
 maman|Chacune a pris sa part, à sa taille.
 papa|L'eau a tenu jusqu'au bout.
 narrateur|La clochette rentre, encore salée.
-narrateur|Mila lisse un coquillage, tout doux.
-copine|Il a bien roulé.
+narrateur|Mila lisse le phare, tout doux.
+copine|Il a bien tenu.
 narrateur|La vague reprend son calme, déjà.</t>
         </is>
       </c>
@@ -6392,12 +6391,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La clochette rentre, encore salée. Un peu de sable reste au rebord. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
+          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La clochette rentre, encore salée. Le phare veille, encore salé. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La clochette rentre, encore salée. Un peu de sable reste au rebord. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
+          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La clochette rentre, encore salée. Le phare veille, encore salé. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6538,7 +6537,7 @@
 papa|Vous avez demandé, rien de plus.
 maman|Mes élastiques rentrent dans la poche.
 narrateur|La clochette rentre, encore salée.
-narrateur|Un peu de sable reste au rebord.
+narrateur|Le phare veille, encore salé.
 enfant-f|Les coquillages sont à nous.
 narrateur|La mer sent encore le vent d'hier.</t>
         </is>
@@ -7670,12 +7669,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Sarah essuie, puis reprend l'anse du seau. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
+          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Puis elle reprend l'anse du seau. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Sarah essuie, puis reprend l'anse du seau. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
+          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Puis elle reprend l'anse du seau. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7813,7 +7812,7 @@
           <t>enfant-f|Maman, le torchon, s'il te plaît.
 maman|Tiens, tout doux, sur les verres.
 narrateur|Sarah frotte un rond, puis un autre.
-narrateur|Sarah essuie, puis reprend l'anse du seau.
+narrateur|Puis elle reprend l'anse du seau.
 copine|Je vois les coquillages !
 enfant-f|Le rose est à toi, maintenant.
 narrateur|Les lunettes rendent le rocher tout net.
@@ -7845,12 +7844,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. Le seau bleu sèche près de la porte. Une goutte reste sur un coquillage, ronde. On rentre, Sarah. La jetée redevient calme.</t>
+          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. Le seau bleu sèche près de la porte. Le phare tient sur la jetée. On rentre, Sarah. La jetée redevient calme.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. Le seau bleu sèche près de la porte. Une goutte reste sur un coquillage, ronde. On rentre, Sarah. La jetée redevient calme.</t>
+          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. Le seau bleu sèche près de la porte. Le phare tient sur la jetée. On rentre, Sarah. La jetée redevient calme.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7991,7 +7990,7 @@
 papa|Vous avez bâti, chacune avec sa vue.
 maman|Le bois sèche déjà, tout doux.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Une goutte reste sur un coquillage, ronde.
+narrateur|Le phare tient sur la jetée.
 enfant-f|On rentre, Sarah.
 narrateur|La jetée redevient calme.</t>
         </is>
@@ -8195,12 +8194,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. Le seau bleu sèche près de la porte. Une ombre de coquillage reste au fond. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
+          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. Le seau bleu sèche près de la porte. Le phare tient, encore un peu flou. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. Le seau bleu sèche près de la porte. Une ombre de coquillage reste au fond. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
+          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. Le seau bleu sèche près de la porte. Le phare tient, encore un peu flou. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8341,7 +8340,7 @@
 papa|Les verres flous n'ont pas arrêté le phare.
 maman|La jetée se tait, enfin.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Une ombre de coquillage reste au fond.
+narrateur|Le phare tient, encore un peu flou.
 enfant-f|À demain, le rocher.
 narrateur|Le rebord redevient tiède, déjà.</t>
         </is>
@@ -8545,12 +8544,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. Le seau bleu sèche près de la porte. Mila souffle sur un coquillage, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
+          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. Le seau bleu sèche près de la porte. Mila souffle sur le phare, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. Le seau bleu sèche près de la porte. Mila souffle sur un coquillage, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
+          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. Le seau bleu sèche près de la porte. Mila souffle sur le phare, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8691,7 +8690,7 @@
 maman|Le pas en arrière a rendu les coquillages.
 papa|Vous avez laissé le temps aux lunettes.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Mila souffle sur un coquillage, tout léger.
+narrateur|Mila souffle sur le phare, tout léger.
 copine|Il brille encore.
 narrateur|Le bois reprend, plus loin.</t>
         </is>
@@ -9266,12 +9265,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. Le seau bleu sèche près de la porte. Une mèche sèche contre le col, tout calme. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
+          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. Le seau bleu sèche près de la porte. Le phare tient sur la dune. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. Le seau bleu sèche près de la porte. Une mèche sèche contre le col, tout calme. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
+          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. Le seau bleu sèche près de la porte. Le phare tient sur la dune. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9412,7 +9411,7 @@
 papa|Chacune a eu sa hauteur, sous le vent.
 maman|Le sable sèche déjà.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Une mèche sèche contre le col, tout calme.
+narrateur|Le phare tient sur la dune.
 enfant-f|On rentre, la dune reste.
 narrateur|Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
@@ -9616,12 +9615,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. Le seau bleu sèche près de la porte. Mila souffle dessus, tout léger. Elle part. Le sel s'efface déjà du sable.</t>
+          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. Le seau bleu sèche près de la porte. Le phare tient, encore salé. Il reste. Le sel s'efface déjà du sable.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. Le seau bleu sèche près de la porte. Mila souffle dessus, tout léger. Elle part. Le sel s'efface déjà du sable.</t>
+          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. Le seau bleu sèche près de la porte. Le phare tient, encore salé. Il reste. Le sel s'efface déjà du sable.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9762,8 +9761,8 @@
 maman|L'eau des cheveux s'en est allée.
 papa|La dune vous rend le silence.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Mila souffle dessus, tout léger.
-copine|Elle part.
+narrateur|Le phare tient, encore salé.
+copine|Il reste.
 narrateur|Le sel s'efface déjà du sable.</t>
         </is>
       </c>
@@ -9966,12 +9965,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. Le seau bleu sèche près de la porte. Un rebord vide attend, tout bas. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
+          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. Le seau bleu sèche près de la porte. Le phare reste, tout petit. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. Le seau bleu sèche près de la porte. Un rebord vide attend, tout bas. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
+          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. Le seau bleu sèche près de la porte. Le phare reste, tout petit. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10112,7 +10111,7 @@
 papa|Vous avez bâti avec ce que vous aviez.
 maman|Les cheveux n'avaient plus besoin d'être pris.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Un rebord vide attend, tout bas.
+narrateur|Le phare reste, tout petit.
 enfant-f|On se dit au revoir, dune.
 narrateur|Les chaussons glissent vers la maison.</t>
         </is>
@@ -10687,12 +10686,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. Le seau bleu sèche près de la porte. Un coquillage rose reste sur le bois. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
+          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. Le seau bleu sèche près de la porte. Le phare tient dans l'écume. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. Le seau bleu sèche près de la porte. Un coquillage rose reste sur le bois. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
+          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. Le seau bleu sèche près de la porte. Le phare tient dans l'écume. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10833,7 +10832,7 @@
 papa|Les manches ont laissé les coquillages passer.
 maman|L'écume redevient de l'eau, tout simple.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Un coquillage rose reste sur le bois.
+narrateur|Le phare tient dans l'écume.
 enfant-f|On rentre, Sarah.
 narrateur|L'écume reprend sa forme, tout lente.</t>
         </is>
@@ -11037,12 +11036,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. Le seau bleu sèche près de la porte. Mila lisse un coquillage, tout doux. Il a bien roulé. La vague reprend son calme, déjà.</t>
+          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. Le seau bleu sèche près de la porte. Mila lisse le phare, tout doux. Il a bien tenu. La vague reprend son calme, déjà.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. Le seau bleu sèche près de la porte. Mila lisse un coquillage, tout doux. Il a bien roulé. La vague reprend son calme, déjà.</t>
+          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. Le seau bleu sèche près de la porte. Mila lisse le phare, tout doux. Il a bien tenu. La vague reprend son calme, déjà.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11183,8 +11182,8 @@
 maman|Chacune a pris sa part, à sa taille.
 papa|L'eau a tenu jusqu'au bout.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Mila lisse un coquillage, tout doux.
-copine|Il a bien roulé.
+narrateur|Mila lisse le phare, tout doux.
+copine|Il a bien tenu.
 narrateur|La vague reprend son calme, déjà.</t>
         </is>
       </c>
@@ -11387,12 +11386,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. Le seau bleu sèche près de la porte. Un peu de sable reste au rebord. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
+          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. Le seau bleu sèche près de la porte. Le phare veille, encore salé. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. Le seau bleu sèche près de la porte. Un peu de sable reste au rebord. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
+          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. Le seau bleu sèche près de la porte. Le phare veille, encore salé. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11533,7 +11532,7 @@
 papa|Vous avez demandé, rien de plus.
 maman|Mes élastiques rentrent dans la poche.
 narrateur|Le seau bleu sèche près de la porte.
-narrateur|Un peu de sable reste au rebord.
+narrateur|Le phare veille, encore salé.
 enfant-f|Les coquillages sont à nous.
 narrateur|La mer sent encore le vent d'hier.</t>
         </is>
@@ -12667,12 +12666,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Sarah essuie, puis reprend le manche de la pelle. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
+          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Puis elle reprend le manche de la pelle. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Sarah essuie, puis reprend le manche de la pelle. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
+          <t>Maman, le torchon, s'il te plaît. Tiens, tout doux, sur les verres. Sarah frotte un rond, puis un autre. Puis elle reprend le manche de la pelle. Je vois les coquillages ! Le rose est à toi, maintenant. Les lunettes rendent le rocher tout net. Vous bâtissez, chacune avec ce qu'elle a. Le torchon a rendu la jetée.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12810,7 +12809,7 @@
           <t>enfant-f|Maman, le torchon, s'il te plaît.
 maman|Tiens, tout doux, sur les verres.
 narrateur|Sarah frotte un rond, puis un autre.
-narrateur|Sarah essuie, puis reprend le manche de la pelle.
+narrateur|Puis elle reprend le manche de la pelle.
 copine|Je vois les coquillages !
 enfant-f|Le rose est à toi, maintenant.
 narrateur|Les lunettes rendent le rocher tout net.
@@ -12842,12 +12841,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La pelle jaune retrouve le sac. Une goutte reste sur un coquillage, ronde. On rentre, Sarah. La jetée redevient calme.</t>
+          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La pelle jaune retrouve le sac. Le phare tient sur la jetée. On rentre, Sarah. La jetée redevient calme.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La pelle jaune retrouve le sac. Une goutte reste sur un coquillage, ronde. On rentre, Sarah. La jetée redevient calme.</t>
+          <t>La jetée sent encore le torchon tiède. J'ai vu le coquillage, tout net. Tes lunettes ont trouvé le rose. Vous avez bâti, chacune avec sa vue. Le bois sèche déjà, tout doux. La pelle jaune retrouve le sac. Le phare tient sur la jetée. On rentre, Sarah. La jetée redevient calme.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12988,7 +12987,7 @@
 papa|Vous avez bâti, chacune avec sa vue.
 maman|Le bois sèche déjà, tout doux.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Une goutte reste sur un coquillage, ronde.
+narrateur|Le phare tient sur la jetée.
 enfant-f|On rentre, Sarah.
 narrateur|La jetée redevient calme.</t>
         </is>
@@ -13192,12 +13191,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La pelle jaune retrouve le sac. Une ombre de coquillage reste au fond. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
+          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La pelle jaune retrouve le sac. Le phare tient, encore un peu flou. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La pelle jaune retrouve le sac. Une ombre de coquillage reste au fond. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
+          <t>Sur le bois, l'air est encore un peu chaud. Tu as touché, moi j'ai dit où. Mes mains ont vu le rose. Les verres flous n'ont pas arrêté le phare. La jetée se tait, enfin. La pelle jaune retrouve le sac. Le phare tient, encore un peu flou. À demain, le rocher. Le rebord redevient tiède, déjà.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13338,7 +13337,7 @@
 papa|Les verres flous n'ont pas arrêté le phare.
 maman|La jetée se tait, enfin.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Une ombre de coquillage reste au fond.
+narrateur|Le phare tient, encore un peu flou.
 enfant-f|À demain, le rocher.
 narrateur|Le rebord redevient tiède, déjà.</t>
         </is>
@@ -13542,12 +13541,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La pelle jaune retrouve le sac. Mila souffle sur un coquillage, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
+          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La pelle jaune retrouve le sac. Mila souffle sur le phare, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La pelle jaune retrouve le sac. Mila souffle sur un coquillage, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
+          <t>Un filet d'air sec reste près de la jetée. L'eau est partie, tout seule. On a attendu le verre clair. Le pas en arrière a rendu les coquillages. Vous avez laissé le temps aux lunettes. La pelle jaune retrouve le sac. Mila souffle sur le phare, tout léger. Il brille encore. Le bois reprend, plus loin.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13688,7 +13687,7 @@
 maman|Le pas en arrière a rendu les coquillages.
 papa|Vous avez laissé le temps aux lunettes.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Mila souffle sur un coquillage, tout léger.
+narrateur|Mila souffle sur le phare, tout léger.
 copine|Il brille encore.
 narrateur|Le bois reprend, plus loin.</t>
         </is>
@@ -14088,12 +14087,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On met le bandeau, plus haut. Mes cheveux restent en arrière, alors. Mila ouvre la pelle, hors des mèches. Maman noue le bandeau, tout doux. Les mèches de Sarah tiennent, libres. Tu peux te pencher, maintenant. Le vent ne m'attrape plus. Chacune a sa hauteur, sur la dune. Les cheveux ont eu leur place.</t>
+          <t>On met le bandeau, plus haut. Mes cheveux restent en arrière, alors. Mila pose la pelle, hors des mèches. Maman noue le bandeau, tout doux. Les mèches de Sarah tiennent, libres. Tu peux te pencher, maintenant. Le vent ne m'attrape plus. Chacune a sa hauteur, sur la dune. Les cheveux ont eu leur place.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>On met le bandeau, plus haut. Mes cheveux restent en arrière, alors. Mila ouvre la pelle, hors des mèches. Maman noue le bandeau, tout doux. Les mèches de Sarah tiennent, libres. Tu peux te pencher, maintenant. Le vent ne m'attrape plus. Chacune a sa hauteur, sur la dune. Les cheveux ont eu leur place.</t>
+          <t>On met le bandeau, plus haut. Mes cheveux restent en arrière, alors. Mila pose la pelle, hors des mèches. Maman noue le bandeau, tout doux. Les mèches de Sarah tiennent, libres. Tu peux te pencher, maintenant. Le vent ne m'attrape plus. Chacune a sa hauteur, sur la dune. Les cheveux ont eu leur place.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14230,7 +14229,7 @@
         <is>
           <t>enfant-f|On met le bandeau, plus haut.
 copine|Mes cheveux restent en arrière, alors.
-narrateur|Mila ouvre la pelle, hors des mèches.
+narrateur|Mila pose la pelle, hors des mèches.
 narrateur|Maman noue le bandeau, tout doux.
 narrateur|Les mèches de Sarah tiennent, libres.
 enfant-f|Tu peux te pencher, maintenant.
@@ -14263,12 +14262,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La pelle jaune retrouve le sac. Une mèche sèche contre le col, tout calme. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
+          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La pelle jaune retrouve le sac. Le phare tient sur la dune. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La pelle jaune retrouve le sac. Une mèche sèche contre le col, tout calme. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
+          <t>La dune garde encore un peu d'ombre. Le bandeau était trop bas, d'abord. Mes cheveux sont restés libres. Chacune a eu sa hauteur, sous le vent. Le sable sèche déjà. La pelle jaune retrouve le sac. Le phare tient sur la dune. On rentre, la dune reste. Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14409,7 +14408,7 @@
 papa|Chacune a eu sa hauteur, sous le vent.
 maman|Le sable sèche déjà.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Une mèche sèche contre le col, tout calme.
+narrateur|Le phare tient sur la dune.
 enfant-f|On rentre, la dune reste.
 narrateur|Un brin d'herbe reprend sa place, tout bas.</t>
         </is>
@@ -14438,12 +14437,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>La serviette, maman ? Frotte, tout doux, pas trop fort. Sarah essuie une mèche, puis une autre. La pelle attend, le temps d'un frottement. Elles sont plus légères ! On ouvre la pelle, maintenant. Le vent pousse, sans emporter de cheveu. Vous avez laissé l'eau des cheveux. La dune sent encore le sel.</t>
+          <t>La serviette, maman ? Frotte, tout doux, pas trop fort. Sarah essuie une mèche, puis une autre. La pelle attend, le temps d'un frottement. Elles sont plus légères ! On pose la pelle, maintenant. Le vent pousse, sans emporter de cheveu. Vous avez laissé l'eau des cheveux. La dune sent encore le sel.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>La serviette, maman ? Frotte, tout doux, pas trop fort. Sarah essuie une mèche, puis une autre. La pelle attend, le temps d'un frottement. Elles sont plus légères ! On ouvre la pelle, maintenant. Le vent pousse, sans emporter de cheveu. Vous avez laissé l'eau des cheveux. La dune sent encore le sel.</t>
+          <t>La serviette, maman ? Frotte, tout doux, pas trop fort. Sarah essuie une mèche, puis une autre. La pelle attend, le temps d'un frottement. Elles sont plus légères ! On pose la pelle, maintenant. Le vent pousse, sans emporter de cheveu. Vous avez laissé l'eau des cheveux. La dune sent encore le sel.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14583,7 +14582,7 @@
 narrateur|Sarah essuie une mèche, puis une autre.
 narrateur|La pelle attend, le temps d'un frottement.
 copine|Elles sont plus légères !
-enfant-f|On ouvre la pelle, maintenant.
+enfant-f|On pose la pelle, maintenant.
 narrateur|Le vent pousse, sans emporter de cheveu.
 papa|Vous avez laissé l'eau des cheveux.
 maman|La dune sent encore le sel.</t>
@@ -14613,12 +14612,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La pelle jaune retrouve le sac. Mila souffle dessus, tout léger. Elle part. Le sel s'efface déjà du sable.</t>
+          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La pelle jaune retrouve le sac. Le phare tient, encore salé. Il reste. Le sel s'efface déjà du sable.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La pelle jaune retrouve le sac. Mila souffle dessus, tout léger. Elle part. Le sel s'efface déjà du sable.</t>
+          <t>La serviette sent encore le sel. Tu as frotté, tout doux. Puis on a bâti, sans emporter de cheveu. L'eau des cheveux s'en est allée. La dune vous rend le silence. La pelle jaune retrouve le sac. Le phare tient, encore salé. Il reste. Le sel s'efface déjà du sable.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14759,8 +14758,8 @@
 maman|L'eau des cheveux s'en est allée.
 papa|La dune vous rend le silence.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Mila souffle dessus, tout léger.
-copine|Elle part.
+narrateur|Le phare tient, encore salé.
+copine|Il reste.
 narrateur|Le sel s'efface déjà du sable.</t>
         </is>
       </c>
@@ -14788,12 +14787,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Tu tiens le seau, moi je pose. Mes mains font le bord, alors. Sarah tient le seau, Mila ouvre la pelle. Les coquillages tombent quand Sarah recule. Ils s'arrêtent quand elle avance. C'est toi le seau vivant, Sarah ! Et toi les coquillages. Vous bâtissez avec ce que vous avez. Les cheveux n'ont plus besoin du vent.</t>
+          <t>Tu tiens le seau, moi je pose. Mes mains font le bord, alors. Sarah tient le seau, Mila pose la pelle. Les coquillages tombent quand Sarah recule. Ils s'arrêtent quand elle avance. C'est toi le seau vivant, Sarah ! Et toi les coquillages. Vous bâtissez avec ce que vous avez. Les cheveux n'ont plus besoin du vent.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Tu tiens le seau, moi je pose. Mes mains font le bord, alors. Sarah tient le seau, Mila ouvre la pelle. Les coquillages tombent quand Sarah recule. Ils s'arrêtent quand elle avance. C'est toi le seau vivant, Sarah ! Et toi les coquillages. Vous bâtissez avec ce que vous avez. Les cheveux n'ont plus besoin du vent.</t>
+          <t>Tu tiens le seau, moi je pose. Mes mains font le bord, alors. Sarah tient le seau, Mila pose la pelle. Les coquillages tombent quand Sarah recule. Ils s'arrêtent quand elle avance. C'est toi le seau vivant, Sarah ! Et toi les coquillages. Vous bâtissez avec ce que vous avez. Les cheveux n'ont plus besoin du vent.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14930,7 +14929,7 @@
         <is>
           <t>enfant-f|Tu tiens le seau, moi je pose.
 copine|Mes mains font le bord, alors.
-narrateur|Sarah tient le seau, Mila ouvre la pelle.
+narrateur|Sarah tient le seau, Mila pose la pelle.
 narrateur|Les coquillages tombent quand Sarah recule.
 narrateur|Ils s'arrêtent quand elle avance.
 enfant-f|C'est toi le seau vivant, Sarah !
@@ -14963,12 +14962,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La pelle jaune retrouve le sac. Un rebord vide attend, tout bas. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
+          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La pelle jaune retrouve le sac. Le phare reste, tout petit. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La pelle jaune retrouve le sac. Un rebord vide attend, tout bas. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
+          <t>Les mains de Sarah gardent encore le pli du seau. Tu étais le seau vivant. Toi les coquillages, moi le bord. Vous avez bâti avec ce que vous aviez. Les cheveux n'avaient plus besoin d'être pris. La pelle jaune retrouve le sac. Le phare reste, tout petit. On se dit au revoir, dune. Les chaussons glissent vers la maison.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15109,7 +15108,7 @@
 papa|Vous avez bâti avec ce que vous aviez.
 maman|Les cheveux n'avaient plus besoin d'être pris.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Un rebord vide attend, tout bas.
+narrateur|Le phare reste, tout petit.
 enfant-f|On se dit au revoir, dune.
 narrateur|Les chaussons glissent vers la maison.</t>
         </is>
@@ -15684,12 +15683,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La pelle jaune retrouve le sac. Un coquillage rose reste sur le bois. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
+          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La pelle jaune retrouve le sac. Le phare tient dans l'écume. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La pelle jaune retrouve le sac. Un coquillage rose reste sur le bois. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
+          <t>Deux rouleaux de manches tiennent encore. Tes mains sont sorties du ciré. Le coquillage n'était plus avalé. Les manches ont laissé les coquillages passer. L'écume redevient de l'eau, tout simple. La pelle jaune retrouve le sac. Le phare tient dans l'écume. On rentre, Sarah. L'écume reprend sa forme, tout lente.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15830,7 +15829,7 @@
 papa|Les manches ont laissé les coquillages passer.
 maman|L'écume redevient de l'eau, tout simple.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Un coquillage rose reste sur le bois.
+narrateur|Le phare tient dans l'écume.
 enfant-f|On rentre, Sarah.
 narrateur|L'écume reprend sa forme, tout lente.</t>
         </is>
@@ -16034,12 +16033,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La pelle jaune retrouve le sac. Mila lisse un coquillage, tout doux. Il a bien roulé. La vague reprend son calme, déjà.</t>
+          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La pelle jaune retrouve le sac. Mila lisse le phare, tout doux. Il a bien tenu. La vague reprend son calme, déjà.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La pelle jaune retrouve le sac. Mila lisse un coquillage, tout doux. Il a bien roulé. La vague reprend son calme, déjà.</t>
+          <t>Une goutte tombe encore d'une manche. Tu tenais la pelle, moi le bord. Tes manches bougeaient seulement le tissu. Chacune a pris sa part, à sa taille. L'eau a tenu jusqu'au bout. La pelle jaune retrouve le sac. Mila lisse le phare, tout doux. Il a bien tenu. La vague reprend son calme, déjà.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16180,8 +16179,8 @@
 maman|Chacune a pris sa part, à sa taille.
 papa|L'eau a tenu jusqu'au bout.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Mila lisse un coquillage, tout doux.
-copine|Il a bien roulé.
+narrateur|Mila lisse le phare, tout doux.
+copine|Il a bien tenu.
 narrateur|La vague reprend son calme, déjà.</t>
         </is>
       </c>
@@ -16384,12 +16383,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La pelle jaune retrouve le sac. Un peu de sable reste au rebord. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
+          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La pelle jaune retrouve le sac. Le phare veille, encore salé. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La pelle jaune retrouve le sac. Un peu de sable reste au rebord. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
+          <t>Deux élastiques veillent encore aux poignets. On a demandé, et ça tenait. Mes mains étaient nues, pour les coquillages. Vous avez demandé, rien de plus. Mes élastiques rentrent dans la poche. La pelle jaune retrouve le sac. Le phare veille, encore salé. Les coquillages sont à nous. La mer sent encore le vent d'hier.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16530,7 +16529,7 @@
 papa|Vous avez demandé, rien de plus.
 maman|Mes élastiques rentrent dans la poche.
 narrateur|La pelle jaune retrouve le sac.
-narrateur|Un peu de sable reste au rebord.
+narrateur|Le phare veille, encore salé.
 enfant-f|Les coquillages sont à nous.
 narrateur|La mer sent encore le vent d'hier.</t>
         </is>
@@ -16553,7 +16552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16652,6 +16651,20 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>